<commit_message>
Completed step 5 by writing all the unit tests in test_investment_account.py file..
</commit_message>
<xml_diff>
--- a/tests/A02_pixell_test_plan_investment_account.xlsx
+++ b/tests/A02_pixell_test_plan_investment_account.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Surmeet Kaur\Documents\intermediate_software_development\activities\project\isd_project\tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{126DF315-61D0-40A3-B930-F38B2149B7D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A9229CC-404A-4ACA-AF1D-B56642E3B215}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{8D9DD509-55B1-455D-8036-16809AD15960}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{8D9DD509-55B1-455D-8036-16809AD15960}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -267,12 +267,6 @@
     <t>Set to 2.55</t>
   </si>
   <si>
-    <t>Date Created: 2026-01-01 Management Fee: Waived Account Type: Investment</t>
-  </si>
-  <si>
-    <t>Date Created: 2019-01-01 Management Fee: $1.99 Account Type: Investment</t>
-  </si>
-  <si>
     <t>12345678
 25
 900.2
@@ -283,21 +277,27 @@
     <t>12345678
 25
 900.2
-date(2026,01,01)
+date(2016,02,15)
 1.99</t>
   </si>
   <si>
     <t>12345678
 25
 900.2
-date(2019,01,01)
+date(2014,02,15)
 1.99</t>
+  </si>
+  <si>
+    <t>Date Created: 2014-02-15 Management Fee: Waived Account Type: Investment</t>
+  </si>
+  <si>
+    <t>Date Created: 2016-02-15 Management Fee: $1.99 Account Type: Investment</t>
   </si>
   <si>
     <t>12345678
 25
 900.2
-date(2015,02,14)
+date(2015,02,15)
 1.99</t>
   </si>
 </sst>
@@ -879,8 +879,8 @@
     <tableColumn id="2" xr3:uid="{1904C92F-9639-4229-AA4E-4C4DEAF21EEE}" name="Method being Tested" dataDxfId="4"/>
     <tableColumn id="3" xr3:uid="{4E480EB6-99FB-4F51-98B5-D5BE13327E8C}" name="Condition being Tested" dataDxfId="3"/>
     <tableColumn id="4" xr3:uid="{5381561B-09C5-439D-999E-CD8E013F9561}" name="Preconditions" dataDxfId="2"/>
-    <tableColumn id="5" xr3:uid="{645704DE-22F5-4239-BEB6-F4252A1F2823}" name="Method Inputs" dataDxfId="0"/>
-    <tableColumn id="6" xr3:uid="{101F480E-86C3-4E60-AA1E-2FCAD389E35F}" name="Expected Result" dataDxfId="1"/>
+    <tableColumn id="5" xr3:uid="{645704DE-22F5-4239-BEB6-F4252A1F2823}" name="Method Inputs" dataDxfId="1"/>
+    <tableColumn id="6" xr3:uid="{101F480E-86C3-4E60-AA1E-2FCAD389E35F}" name="Expected Result" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium16" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1282,7 +1282,7 @@
         <v>22</v>
       </c>
       <c r="F7" s="12" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="G7" s="12" t="s">
         <v>23</v>
@@ -1319,7 +1319,7 @@
         <v>14</v>
       </c>
       <c r="E9" s="12" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F9" s="13" t="s">
         <v>22</v>
@@ -1359,7 +1359,7 @@
         <v>15</v>
       </c>
       <c r="E11" s="12" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="F11" s="13" t="s">
         <v>22</v>
@@ -1379,13 +1379,13 @@
         <v>16</v>
       </c>
       <c r="E12" s="12" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F12" s="13" t="s">
         <v>22</v>
       </c>
       <c r="G12" s="13" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
     </row>
     <row r="13" spans="2:7" ht="71.400000000000006" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -1399,13 +1399,13 @@
         <v>17</v>
       </c>
       <c r="E13" s="12" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="F13" s="13" t="s">
         <v>22</v>
       </c>
       <c r="G13" s="13" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
     </row>
     <row r="14" spans="2:7" ht="31.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">

</xml_diff>